<commit_message>
Upgrade detection rules to V2 specification (Sigma normalization & OCSF mapping)
</commit_message>
<xml_diff>
--- a/window-correlation-rules/ocsf_mapped_new_sprint.xlsx
+++ b/window-correlation-rules/ocsf_mapped_new_sprint.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N376"/>
+  <dimension ref="A1:O376"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -499,6 +499,11 @@
           <t xml:space="preserve">updated or not </t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>v2 version done</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -571,6 +576,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -643,6 +649,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -715,6 +722,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -787,6 +795,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -859,6 +868,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -931,6 +941,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1003,6 +1014,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1075,6 +1087,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1147,6 +1160,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1219,6 +1233,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1291,6 +1306,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1363,6 +1379,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1435,6 +1452,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1507,6 +1525,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1579,6 +1598,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1646,7 +1666,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr"/>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1714,7 +1739,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr"/>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1782,7 +1812,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr"/>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1850,7 +1885,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr"/>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1918,7 +1958,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr"/>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1986,7 +2031,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr"/>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2054,7 +2104,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr"/>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2122,7 +2177,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr"/>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2190,7 +2250,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr"/>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2258,7 +2323,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr"/>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2327,6 +2397,7 @@
         </is>
       </c>
       <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2395,6 +2466,7 @@
         </is>
       </c>
       <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2463,6 +2535,7 @@
         </is>
       </c>
       <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2531,6 +2604,7 @@
         </is>
       </c>
       <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2599,6 +2673,7 @@
         </is>
       </c>
       <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2667,6 +2742,7 @@
         </is>
       </c>
       <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2735,6 +2811,7 @@
         </is>
       </c>
       <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2803,6 +2880,7 @@
         </is>
       </c>
       <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2871,6 +2949,7 @@
         </is>
       </c>
       <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2939,6 +3018,7 @@
         </is>
       </c>
       <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3007,6 +3087,7 @@
         </is>
       </c>
       <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3079,6 +3160,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3147,6 +3229,7 @@
         </is>
       </c>
       <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3215,6 +3298,7 @@
         </is>
       </c>
       <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3283,6 +3367,7 @@
         </is>
       </c>
       <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3351,6 +3436,7 @@
         </is>
       </c>
       <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3419,6 +3505,7 @@
         </is>
       </c>
       <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3487,6 +3574,7 @@
         </is>
       </c>
       <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3555,6 +3643,7 @@
         </is>
       </c>
       <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3623,6 +3712,7 @@
         </is>
       </c>
       <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3691,6 +3781,7 @@
         </is>
       </c>
       <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3759,6 +3850,7 @@
         </is>
       </c>
       <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3827,6 +3919,7 @@
         </is>
       </c>
       <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3895,6 +3988,7 @@
         </is>
       </c>
       <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3963,6 +4057,7 @@
         </is>
       </c>
       <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4031,6 +4126,7 @@
         </is>
       </c>
       <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4099,6 +4195,7 @@
         </is>
       </c>
       <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4167,6 +4264,7 @@
         </is>
       </c>
       <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4235,6 +4333,7 @@
         </is>
       </c>
       <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4303,6 +4402,7 @@
         </is>
       </c>
       <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4371,6 +4471,7 @@
         </is>
       </c>
       <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4439,6 +4540,7 @@
         </is>
       </c>
       <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4507,6 +4609,7 @@
         </is>
       </c>
       <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4566,7 +4669,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -4575,6 +4678,7 @@
         </is>
       </c>
       <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4634,7 +4738,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
@@ -4643,6 +4747,7 @@
         </is>
       </c>
       <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4702,7 +4807,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
@@ -4711,6 +4816,7 @@
         </is>
       </c>
       <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4770,7 +4876,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
@@ -4779,6 +4885,7 @@
         </is>
       </c>
       <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4838,7 +4945,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
@@ -4847,6 +4954,7 @@
         </is>
       </c>
       <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4906,7 +5014,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -4915,6 +5023,7 @@
         </is>
       </c>
       <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4974,7 +5083,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
@@ -4983,6 +5092,7 @@
         </is>
       </c>
       <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5042,7 +5152,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
@@ -5051,6 +5161,7 @@
         </is>
       </c>
       <c r="N67" t="inlineStr"/>
+      <c r="O67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5110,7 +5221,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
@@ -5119,6 +5230,7 @@
         </is>
       </c>
       <c r="N68" t="inlineStr"/>
+      <c r="O68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5178,7 +5290,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
@@ -5187,6 +5299,7 @@
         </is>
       </c>
       <c r="N69" t="inlineStr"/>
+      <c r="O69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5246,7 +5359,7 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
@@ -5255,6 +5368,7 @@
         </is>
       </c>
       <c r="N70" t="inlineStr"/>
+      <c r="O70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5314,7 +5428,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
@@ -5323,6 +5437,7 @@
         </is>
       </c>
       <c r="N71" t="inlineStr"/>
+      <c r="O71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -5382,7 +5497,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
@@ -5391,6 +5506,7 @@
         </is>
       </c>
       <c r="N72" t="inlineStr"/>
+      <c r="O72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5450,7 +5566,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
@@ -5459,6 +5575,7 @@
         </is>
       </c>
       <c r="N73" t="inlineStr"/>
+      <c r="O73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -5518,7 +5635,7 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
@@ -5527,6 +5644,7 @@
         </is>
       </c>
       <c r="N74" t="inlineStr"/>
+      <c r="O74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5586,7 +5704,7 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
@@ -5595,6 +5713,7 @@
         </is>
       </c>
       <c r="N75" t="inlineStr"/>
+      <c r="O75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5654,7 +5773,7 @@
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
@@ -5663,6 +5782,7 @@
         </is>
       </c>
       <c r="N76" t="inlineStr"/>
+      <c r="O76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -5722,7 +5842,7 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
@@ -5731,6 +5851,7 @@
         </is>
       </c>
       <c r="N77" t="inlineStr"/>
+      <c r="O77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -5799,6 +5920,7 @@
         </is>
       </c>
       <c r="N78" t="inlineStr"/>
+      <c r="O78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -5867,6 +5989,7 @@
         </is>
       </c>
       <c r="N79" t="inlineStr"/>
+      <c r="O79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -5935,6 +6058,7 @@
         </is>
       </c>
       <c r="N80" t="inlineStr"/>
+      <c r="O80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -6003,6 +6127,7 @@
         </is>
       </c>
       <c r="N81" t="inlineStr"/>
+      <c r="O81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6071,6 +6196,7 @@
         </is>
       </c>
       <c r="N82" t="inlineStr"/>
+      <c r="O82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -6139,6 +6265,7 @@
         </is>
       </c>
       <c r="N83" t="inlineStr"/>
+      <c r="O83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -6207,6 +6334,7 @@
         </is>
       </c>
       <c r="N84" t="inlineStr"/>
+      <c r="O84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -6275,6 +6403,7 @@
         </is>
       </c>
       <c r="N85" t="inlineStr"/>
+      <c r="O85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6343,6 +6472,7 @@
         </is>
       </c>
       <c r="N86" t="inlineStr"/>
+      <c r="O86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6411,6 +6541,7 @@
         </is>
       </c>
       <c r="N87" t="inlineStr"/>
+      <c r="O87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -6479,6 +6610,7 @@
         </is>
       </c>
       <c r="N88" t="inlineStr"/>
+      <c r="O88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -6547,6 +6679,7 @@
         </is>
       </c>
       <c r="N89" t="inlineStr"/>
+      <c r="O89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -6615,6 +6748,7 @@
         </is>
       </c>
       <c r="N90" t="inlineStr"/>
+      <c r="O90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -6683,6 +6817,7 @@
         </is>
       </c>
       <c r="N91" t="inlineStr"/>
+      <c r="O91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -6751,6 +6886,7 @@
         </is>
       </c>
       <c r="N92" t="inlineStr"/>
+      <c r="O92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -6819,6 +6955,7 @@
         </is>
       </c>
       <c r="N93" t="inlineStr"/>
+      <c r="O93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -6887,6 +7024,7 @@
         </is>
       </c>
       <c r="N94" t="inlineStr"/>
+      <c r="O94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -6955,6 +7093,7 @@
         </is>
       </c>
       <c r="N95" t="inlineStr"/>
+      <c r="O95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -7023,6 +7162,7 @@
         </is>
       </c>
       <c r="N96" t="inlineStr"/>
+      <c r="O96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -7091,6 +7231,7 @@
         </is>
       </c>
       <c r="N97" t="inlineStr"/>
+      <c r="O97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -7159,6 +7300,7 @@
         </is>
       </c>
       <c r="N98" t="inlineStr"/>
+      <c r="O98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -7227,6 +7369,7 @@
         </is>
       </c>
       <c r="N99" t="inlineStr"/>
+      <c r="O99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -7295,6 +7438,7 @@
         </is>
       </c>
       <c r="N100" t="inlineStr"/>
+      <c r="O100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -7363,6 +7507,7 @@
         </is>
       </c>
       <c r="N101" t="inlineStr"/>
+      <c r="O101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -7431,6 +7576,7 @@
         </is>
       </c>
       <c r="N102" t="inlineStr"/>
+      <c r="O102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -7499,6 +7645,7 @@
         </is>
       </c>
       <c r="N103" t="inlineStr"/>
+      <c r="O103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -7567,6 +7714,7 @@
         </is>
       </c>
       <c r="N104" t="inlineStr"/>
+      <c r="O104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -7635,6 +7783,7 @@
         </is>
       </c>
       <c r="N105" t="inlineStr"/>
+      <c r="O105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -7703,6 +7852,7 @@
         </is>
       </c>
       <c r="N106" t="inlineStr"/>
+      <c r="O106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -7771,6 +7921,7 @@
         </is>
       </c>
       <c r="N107" t="inlineStr"/>
+      <c r="O107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -7839,6 +7990,7 @@
         </is>
       </c>
       <c r="N108" t="inlineStr"/>
+      <c r="O108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -7907,6 +8059,7 @@
         </is>
       </c>
       <c r="N109" t="inlineStr"/>
+      <c r="O109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -7975,6 +8128,7 @@
         </is>
       </c>
       <c r="N110" t="inlineStr"/>
+      <c r="O110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -8042,7 +8196,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N111" t="inlineStr"/>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -8110,7 +8269,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N112" t="inlineStr"/>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -8178,7 +8342,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N113" t="inlineStr"/>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -8246,7 +8415,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N114" t="inlineStr"/>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -8314,7 +8488,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N115" t="inlineStr"/>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -8382,7 +8561,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N116" t="inlineStr"/>
+      <c r="N116" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -8450,7 +8634,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N117" t="inlineStr"/>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -8518,7 +8707,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N118" t="inlineStr"/>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -8586,7 +8780,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N119" t="inlineStr"/>
+      <c r="N119" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -8654,7 +8853,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N120" t="inlineStr"/>
+      <c r="N120" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -8722,7 +8926,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N121" t="inlineStr"/>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -8790,7 +8999,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N122" t="inlineStr"/>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -8858,7 +9072,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N123" t="inlineStr"/>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -8926,7 +9145,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N124" t="inlineStr"/>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -8994,7 +9218,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N125" t="inlineStr"/>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -9062,7 +9291,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N126" t="inlineStr"/>
+      <c r="N126" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -9130,7 +9364,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N127" t="inlineStr"/>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -9198,7 +9437,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N128" t="inlineStr"/>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -9267,6 +9511,7 @@
         </is>
       </c>
       <c r="N129" t="inlineStr"/>
+      <c r="O129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -9335,6 +9580,7 @@
         </is>
       </c>
       <c r="N130" t="inlineStr"/>
+      <c r="O130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -9403,6 +9649,7 @@
         </is>
       </c>
       <c r="N131" t="inlineStr"/>
+      <c r="O131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -9471,6 +9718,7 @@
         </is>
       </c>
       <c r="N132" t="inlineStr"/>
+      <c r="O132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -9539,6 +9787,7 @@
         </is>
       </c>
       <c r="N133" t="inlineStr"/>
+      <c r="O133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -9607,6 +9856,7 @@
         </is>
       </c>
       <c r="N134" t="inlineStr"/>
+      <c r="O134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -9675,6 +9925,7 @@
         </is>
       </c>
       <c r="N135" t="inlineStr"/>
+      <c r="O135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -9743,6 +9994,7 @@
         </is>
       </c>
       <c r="N136" t="inlineStr"/>
+      <c r="O136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -9811,6 +10063,7 @@
         </is>
       </c>
       <c r="N137" t="inlineStr"/>
+      <c r="O137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -9879,6 +10132,7 @@
         </is>
       </c>
       <c r="N138" t="inlineStr"/>
+      <c r="O138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -9947,6 +10201,7 @@
         </is>
       </c>
       <c r="N139" t="inlineStr"/>
+      <c r="O139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -10015,6 +10270,7 @@
         </is>
       </c>
       <c r="N140" t="inlineStr"/>
+      <c r="O140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -10083,6 +10339,7 @@
         </is>
       </c>
       <c r="N141" t="inlineStr"/>
+      <c r="O141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -10151,6 +10408,7 @@
         </is>
       </c>
       <c r="N142" t="inlineStr"/>
+      <c r="O142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -10219,6 +10477,7 @@
         </is>
       </c>
       <c r="N143" t="inlineStr"/>
+      <c r="O143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -10287,6 +10546,7 @@
         </is>
       </c>
       <c r="N144" t="inlineStr"/>
+      <c r="O144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -10355,6 +10615,7 @@
         </is>
       </c>
       <c r="N145" t="inlineStr"/>
+      <c r="O145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -10423,6 +10684,7 @@
         </is>
       </c>
       <c r="N146" t="inlineStr"/>
+      <c r="O146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -10491,6 +10753,7 @@
         </is>
       </c>
       <c r="N147" t="inlineStr"/>
+      <c r="O147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -10559,6 +10822,7 @@
         </is>
       </c>
       <c r="N148" t="inlineStr"/>
+      <c r="O148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -10627,6 +10891,7 @@
         </is>
       </c>
       <c r="N149" t="inlineStr"/>
+      <c r="O149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -10695,6 +10960,7 @@
         </is>
       </c>
       <c r="N150" t="inlineStr"/>
+      <c r="O150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -10763,6 +11029,7 @@
         </is>
       </c>
       <c r="N151" t="inlineStr"/>
+      <c r="O151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -10831,6 +11098,7 @@
         </is>
       </c>
       <c r="N152" t="inlineStr"/>
+      <c r="O152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -10899,6 +11167,7 @@
         </is>
       </c>
       <c r="N153" t="inlineStr"/>
+      <c r="O153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -10967,6 +11236,7 @@
         </is>
       </c>
       <c r="N154" t="inlineStr"/>
+      <c r="O154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -11035,6 +11305,7 @@
         </is>
       </c>
       <c r="N155" t="inlineStr"/>
+      <c r="O155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -11103,6 +11374,7 @@
         </is>
       </c>
       <c r="N156" t="inlineStr"/>
+      <c r="O156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -11171,6 +11443,7 @@
         </is>
       </c>
       <c r="N157" t="inlineStr"/>
+      <c r="O157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -11239,6 +11512,7 @@
         </is>
       </c>
       <c r="N158" t="inlineStr"/>
+      <c r="O158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -11307,6 +11581,7 @@
         </is>
       </c>
       <c r="N159" t="inlineStr"/>
+      <c r="O159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -11375,6 +11650,7 @@
         </is>
       </c>
       <c r="N160" t="inlineStr"/>
+      <c r="O160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -11443,6 +11719,7 @@
         </is>
       </c>
       <c r="N161" t="inlineStr"/>
+      <c r="O161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -11511,6 +11788,7 @@
         </is>
       </c>
       <c r="N162" t="inlineStr"/>
+      <c r="O162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -11579,6 +11857,7 @@
         </is>
       </c>
       <c r="N163" t="inlineStr"/>
+      <c r="O163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -11647,6 +11926,7 @@
         </is>
       </c>
       <c r="N164" t="inlineStr"/>
+      <c r="O164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -11715,6 +11995,7 @@
         </is>
       </c>
       <c r="N165" t="inlineStr"/>
+      <c r="O165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -11783,6 +12064,7 @@
         </is>
       </c>
       <c r="N166" t="inlineStr"/>
+      <c r="O166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -11851,6 +12133,7 @@
         </is>
       </c>
       <c r="N167" t="inlineStr"/>
+      <c r="O167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -11919,6 +12202,7 @@
         </is>
       </c>
       <c r="N168" t="inlineStr"/>
+      <c r="O168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -11987,6 +12271,7 @@
         </is>
       </c>
       <c r="N169" t="inlineStr"/>
+      <c r="O169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -12055,6 +12340,7 @@
         </is>
       </c>
       <c r="N170" t="inlineStr"/>
+      <c r="O170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -12123,6 +12409,7 @@
         </is>
       </c>
       <c r="N171" t="inlineStr"/>
+      <c r="O171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -12191,6 +12478,7 @@
         </is>
       </c>
       <c r="N172" t="inlineStr"/>
+      <c r="O172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -12259,6 +12547,7 @@
         </is>
       </c>
       <c r="N173" t="inlineStr"/>
+      <c r="O173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -12327,6 +12616,7 @@
         </is>
       </c>
       <c r="N174" t="inlineStr"/>
+      <c r="O174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -12395,6 +12685,7 @@
         </is>
       </c>
       <c r="N175" t="inlineStr"/>
+      <c r="O175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -12463,6 +12754,7 @@
         </is>
       </c>
       <c r="N176" t="inlineStr"/>
+      <c r="O176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -12531,6 +12823,7 @@
         </is>
       </c>
       <c r="N177" t="inlineStr"/>
+      <c r="O177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -12599,6 +12892,7 @@
         </is>
       </c>
       <c r="N178" t="inlineStr"/>
+      <c r="O178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -12667,6 +12961,7 @@
         </is>
       </c>
       <c r="N179" t="inlineStr"/>
+      <c r="O179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -12735,6 +13030,7 @@
         </is>
       </c>
       <c r="N180" t="inlineStr"/>
+      <c r="O180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -12803,6 +13099,7 @@
         </is>
       </c>
       <c r="N181" t="inlineStr"/>
+      <c r="O181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -12871,6 +13168,7 @@
         </is>
       </c>
       <c r="N182" t="inlineStr"/>
+      <c r="O182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -12939,6 +13237,7 @@
         </is>
       </c>
       <c r="N183" t="inlineStr"/>
+      <c r="O183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -13007,6 +13306,7 @@
         </is>
       </c>
       <c r="N184" t="inlineStr"/>
+      <c r="O184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -13075,6 +13375,7 @@
         </is>
       </c>
       <c r="N185" t="inlineStr"/>
+      <c r="O185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -13143,6 +13444,7 @@
         </is>
       </c>
       <c r="N186" t="inlineStr"/>
+      <c r="O186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -13211,6 +13513,7 @@
         </is>
       </c>
       <c r="N187" t="inlineStr"/>
+      <c r="O187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -13279,6 +13582,7 @@
         </is>
       </c>
       <c r="N188" t="inlineStr"/>
+      <c r="O188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -13347,6 +13651,7 @@
         </is>
       </c>
       <c r="N189" t="inlineStr"/>
+      <c r="O189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -13415,6 +13720,7 @@
         </is>
       </c>
       <c r="N190" t="inlineStr"/>
+      <c r="O190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -13483,6 +13789,7 @@
         </is>
       </c>
       <c r="N191" t="inlineStr"/>
+      <c r="O191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -13551,6 +13858,7 @@
         </is>
       </c>
       <c r="N192" t="inlineStr"/>
+      <c r="O192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -13619,6 +13927,7 @@
         </is>
       </c>
       <c r="N193" t="inlineStr"/>
+      <c r="O193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -13687,6 +13996,7 @@
         </is>
       </c>
       <c r="N194" t="inlineStr"/>
+      <c r="O194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -13755,6 +14065,7 @@
         </is>
       </c>
       <c r="N195" t="inlineStr"/>
+      <c r="O195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -13823,6 +14134,7 @@
         </is>
       </c>
       <c r="N196" t="inlineStr"/>
+      <c r="O196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -13891,6 +14203,7 @@
         </is>
       </c>
       <c r="N197" t="inlineStr"/>
+      <c r="O197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -13959,6 +14272,7 @@
         </is>
       </c>
       <c r="N198" t="inlineStr"/>
+      <c r="O198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -14027,6 +14341,7 @@
         </is>
       </c>
       <c r="N199" t="inlineStr"/>
+      <c r="O199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -14095,6 +14410,7 @@
         </is>
       </c>
       <c r="N200" t="inlineStr"/>
+      <c r="O200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -14163,6 +14479,7 @@
         </is>
       </c>
       <c r="N201" t="inlineStr"/>
+      <c r="O201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -14231,6 +14548,7 @@
         </is>
       </c>
       <c r="N202" t="inlineStr"/>
+      <c r="O202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -14299,6 +14617,7 @@
         </is>
       </c>
       <c r="N203" t="inlineStr"/>
+      <c r="O203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -14367,6 +14686,7 @@
         </is>
       </c>
       <c r="N204" t="inlineStr"/>
+      <c r="O204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -14435,6 +14755,7 @@
         </is>
       </c>
       <c r="N205" t="inlineStr"/>
+      <c r="O205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -14503,6 +14824,7 @@
         </is>
       </c>
       <c r="N206" t="inlineStr"/>
+      <c r="O206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -14571,6 +14893,7 @@
         </is>
       </c>
       <c r="N207" t="inlineStr"/>
+      <c r="O207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -14639,6 +14962,7 @@
         </is>
       </c>
       <c r="N208" t="inlineStr"/>
+      <c r="O208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -14707,6 +15031,7 @@
         </is>
       </c>
       <c r="N209" t="inlineStr"/>
+      <c r="O209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -14775,6 +15100,7 @@
         </is>
       </c>
       <c r="N210" t="inlineStr"/>
+      <c r="O210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -14843,6 +15169,7 @@
         </is>
       </c>
       <c r="N211" t="inlineStr"/>
+      <c r="O211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -14911,6 +15238,7 @@
         </is>
       </c>
       <c r="N212" t="inlineStr"/>
+      <c r="O212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -14979,6 +15307,7 @@
         </is>
       </c>
       <c r="N213" t="inlineStr"/>
+      <c r="O213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -15047,6 +15376,7 @@
         </is>
       </c>
       <c r="N214" t="inlineStr"/>
+      <c r="O214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -15115,6 +15445,7 @@
         </is>
       </c>
       <c r="N215" t="inlineStr"/>
+      <c r="O215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -15183,6 +15514,7 @@
         </is>
       </c>
       <c r="N216" t="inlineStr"/>
+      <c r="O216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -15251,6 +15583,7 @@
         </is>
       </c>
       <c r="N217" t="inlineStr"/>
+      <c r="O217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -15319,6 +15652,7 @@
         </is>
       </c>
       <c r="N218" t="inlineStr"/>
+      <c r="O218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -15387,6 +15721,7 @@
         </is>
       </c>
       <c r="N219" t="inlineStr"/>
+      <c r="O219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -15455,6 +15790,7 @@
         </is>
       </c>
       <c r="N220" t="inlineStr"/>
+      <c r="O220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -15514,7 +15850,7 @@
       </c>
       <c r="L221" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M221" t="inlineStr">
@@ -15522,7 +15858,16 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N221" t="inlineStr"/>
+      <c r="N221" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O221" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -15582,7 +15927,7 @@
       </c>
       <c r="L222" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M222" t="inlineStr">
@@ -15590,7 +15935,16 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N222" t="inlineStr"/>
+      <c r="N222" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O222" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -15650,7 +16004,7 @@
       </c>
       <c r="L223" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M223" t="inlineStr">
@@ -15658,7 +16012,16 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N223" t="inlineStr"/>
+      <c r="N223" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O223" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -15718,7 +16081,7 @@
       </c>
       <c r="L224" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M224" t="inlineStr">
@@ -15726,7 +16089,16 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N224" t="inlineStr"/>
+      <c r="N224" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O224" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -15795,6 +16167,7 @@
         </is>
       </c>
       <c r="N225" t="inlineStr"/>
+      <c r="O225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -15863,6 +16236,7 @@
         </is>
       </c>
       <c r="N226" t="inlineStr"/>
+      <c r="O226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -15931,6 +16305,7 @@
         </is>
       </c>
       <c r="N227" t="inlineStr"/>
+      <c r="O227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -15999,6 +16374,7 @@
         </is>
       </c>
       <c r="N228" t="inlineStr"/>
+      <c r="O228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -16067,6 +16443,7 @@
         </is>
       </c>
       <c r="N229" t="inlineStr"/>
+      <c r="O229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -16135,6 +16512,7 @@
         </is>
       </c>
       <c r="N230" t="inlineStr"/>
+      <c r="O230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -16203,6 +16581,7 @@
         </is>
       </c>
       <c r="N231" t="inlineStr"/>
+      <c r="O231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -16271,6 +16650,7 @@
         </is>
       </c>
       <c r="N232" t="inlineStr"/>
+      <c r="O232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -16339,6 +16719,7 @@
         </is>
       </c>
       <c r="N233" t="inlineStr"/>
+      <c r="O233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -16407,6 +16788,7 @@
         </is>
       </c>
       <c r="N234" t="inlineStr"/>
+      <c r="O234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -16475,6 +16857,7 @@
         </is>
       </c>
       <c r="N235" t="inlineStr"/>
+      <c r="O235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -16543,6 +16926,7 @@
         </is>
       </c>
       <c r="N236" t="inlineStr"/>
+      <c r="O236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -16611,6 +16995,7 @@
         </is>
       </c>
       <c r="N237" t="inlineStr"/>
+      <c r="O237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -16679,6 +17064,7 @@
         </is>
       </c>
       <c r="N238" t="inlineStr"/>
+      <c r="O238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -16747,6 +17133,7 @@
         </is>
       </c>
       <c r="N239" t="inlineStr"/>
+      <c r="O239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -16815,6 +17202,7 @@
         </is>
       </c>
       <c r="N240" t="inlineStr"/>
+      <c r="O240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -16883,6 +17271,7 @@
         </is>
       </c>
       <c r="N241" t="inlineStr"/>
+      <c r="O241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -16951,6 +17340,7 @@
         </is>
       </c>
       <c r="N242" t="inlineStr"/>
+      <c r="O242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -17019,6 +17409,7 @@
         </is>
       </c>
       <c r="N243" t="inlineStr"/>
+      <c r="O243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -17087,6 +17478,7 @@
         </is>
       </c>
       <c r="N244" t="inlineStr"/>
+      <c r="O244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -17155,6 +17547,7 @@
         </is>
       </c>
       <c r="N245" t="inlineStr"/>
+      <c r="O245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -17223,6 +17616,7 @@
         </is>
       </c>
       <c r="N246" t="inlineStr"/>
+      <c r="O246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -17291,6 +17685,7 @@
         </is>
       </c>
       <c r="N247" t="inlineStr"/>
+      <c r="O247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -17359,6 +17754,7 @@
         </is>
       </c>
       <c r="N248" t="inlineStr"/>
+      <c r="O248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -17427,6 +17823,7 @@
         </is>
       </c>
       <c r="N249" t="inlineStr"/>
+      <c r="O249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -17495,6 +17892,7 @@
         </is>
       </c>
       <c r="N250" t="inlineStr"/>
+      <c r="O250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -17563,6 +17961,7 @@
         </is>
       </c>
       <c r="N251" t="inlineStr"/>
+      <c r="O251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -17631,6 +18030,7 @@
         </is>
       </c>
       <c r="N252" t="inlineStr"/>
+      <c r="O252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -17699,6 +18099,7 @@
         </is>
       </c>
       <c r="N253" t="inlineStr"/>
+      <c r="O253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -17767,6 +18168,7 @@
         </is>
       </c>
       <c r="N254" t="inlineStr"/>
+      <c r="O254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -17835,6 +18237,7 @@
         </is>
       </c>
       <c r="N255" t="inlineStr"/>
+      <c r="O255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -17903,6 +18306,7 @@
         </is>
       </c>
       <c r="N256" t="inlineStr"/>
+      <c r="O256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -17971,6 +18375,7 @@
         </is>
       </c>
       <c r="N257" t="inlineStr"/>
+      <c r="O257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -18039,6 +18444,7 @@
         </is>
       </c>
       <c r="N258" t="inlineStr"/>
+      <c r="O258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -18107,6 +18513,7 @@
         </is>
       </c>
       <c r="N259" t="inlineStr"/>
+      <c r="O259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -18175,6 +18582,7 @@
         </is>
       </c>
       <c r="N260" t="inlineStr"/>
+      <c r="O260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -18243,6 +18651,7 @@
         </is>
       </c>
       <c r="N261" t="inlineStr"/>
+      <c r="O261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -18311,6 +18720,7 @@
         </is>
       </c>
       <c r="N262" t="inlineStr"/>
+      <c r="O262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -18379,6 +18789,7 @@
         </is>
       </c>
       <c r="N263" t="inlineStr"/>
+      <c r="O263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -18447,6 +18858,7 @@
         </is>
       </c>
       <c r="N264" t="inlineStr"/>
+      <c r="O264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -18515,6 +18927,7 @@
         </is>
       </c>
       <c r="N265" t="inlineStr"/>
+      <c r="O265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -18583,6 +18996,7 @@
         </is>
       </c>
       <c r="N266" t="inlineStr"/>
+      <c r="O266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -18651,6 +19065,7 @@
         </is>
       </c>
       <c r="N267" t="inlineStr"/>
+      <c r="O267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -18719,6 +19134,7 @@
         </is>
       </c>
       <c r="N268" t="inlineStr"/>
+      <c r="O268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -18787,6 +19203,7 @@
         </is>
       </c>
       <c r="N269" t="inlineStr"/>
+      <c r="O269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -18855,6 +19272,7 @@
         </is>
       </c>
       <c r="N270" t="inlineStr"/>
+      <c r="O270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -18923,6 +19341,7 @@
         </is>
       </c>
       <c r="N271" t="inlineStr"/>
+      <c r="O271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -18991,6 +19410,7 @@
         </is>
       </c>
       <c r="N272" t="inlineStr"/>
+      <c r="O272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -19059,6 +19479,7 @@
         </is>
       </c>
       <c r="N273" t="inlineStr"/>
+      <c r="O273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -19127,6 +19548,7 @@
         </is>
       </c>
       <c r="N274" t="inlineStr"/>
+      <c r="O274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -19195,6 +19617,7 @@
         </is>
       </c>
       <c r="N275" t="inlineStr"/>
+      <c r="O275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -19263,6 +19686,7 @@
         </is>
       </c>
       <c r="N276" t="inlineStr"/>
+      <c r="O276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -19331,6 +19755,7 @@
         </is>
       </c>
       <c r="N277" t="inlineStr"/>
+      <c r="O277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -19399,6 +19824,7 @@
         </is>
       </c>
       <c r="N278" t="inlineStr"/>
+      <c r="O278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -19471,6 +19897,11 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O279" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -19543,6 +19974,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -19615,6 +20047,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -19687,6 +20120,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -19759,6 +20193,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -19831,6 +20266,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O284" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -19903,6 +20339,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O285" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -19975,6 +20412,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O286" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -20047,6 +20485,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O287" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -20119,6 +20558,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O288" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -20191,6 +20631,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O289" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -20263,6 +20704,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -20335,6 +20777,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O291" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -20407,6 +20850,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -20479,6 +20923,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -20551,6 +20996,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -20623,6 +21069,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -20695,6 +21142,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -20767,6 +21215,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O297" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -20839,6 +21288,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O298" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -20911,6 +21361,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -20983,6 +21434,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O300" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -21055,6 +21507,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O301" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -21127,6 +21580,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O302" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -21199,6 +21653,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O303" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -21271,6 +21726,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O304" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -21343,6 +21799,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -21411,6 +21868,7 @@
         </is>
       </c>
       <c r="N306" t="inlineStr"/>
+      <c r="O306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -21479,6 +21937,7 @@
         </is>
       </c>
       <c r="N307" t="inlineStr"/>
+      <c r="O307" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -21547,6 +22006,7 @@
         </is>
       </c>
       <c r="N308" t="inlineStr"/>
+      <c r="O308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -21615,6 +22075,7 @@
         </is>
       </c>
       <c r="N309" t="inlineStr"/>
+      <c r="O309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -21683,6 +22144,7 @@
         </is>
       </c>
       <c r="N310" t="inlineStr"/>
+      <c r="O310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -21751,6 +22213,7 @@
         </is>
       </c>
       <c r="N311" t="inlineStr"/>
+      <c r="O311" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -21819,6 +22282,7 @@
         </is>
       </c>
       <c r="N312" t="inlineStr"/>
+      <c r="O312" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -21887,6 +22351,7 @@
         </is>
       </c>
       <c r="N313" t="inlineStr"/>
+      <c r="O313" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -21955,6 +22420,7 @@
         </is>
       </c>
       <c r="N314" t="inlineStr"/>
+      <c r="O314" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -22023,6 +22489,7 @@
         </is>
       </c>
       <c r="N315" t="inlineStr"/>
+      <c r="O315" t="inlineStr"/>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -22091,6 +22558,7 @@
         </is>
       </c>
       <c r="N316" t="inlineStr"/>
+      <c r="O316" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -22159,6 +22627,7 @@
         </is>
       </c>
       <c r="N317" t="inlineStr"/>
+      <c r="O317" t="inlineStr"/>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -22227,6 +22696,7 @@
         </is>
       </c>
       <c r="N318" t="inlineStr"/>
+      <c r="O318" t="inlineStr"/>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -22295,6 +22765,7 @@
         </is>
       </c>
       <c r="N319" t="inlineStr"/>
+      <c r="O319" t="inlineStr"/>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -22363,6 +22834,7 @@
         </is>
       </c>
       <c r="N320" t="inlineStr"/>
+      <c r="O320" t="inlineStr"/>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -22431,6 +22903,7 @@
         </is>
       </c>
       <c r="N321" t="inlineStr"/>
+      <c r="O321" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -22499,6 +22972,7 @@
         </is>
       </c>
       <c r="N322" t="inlineStr"/>
+      <c r="O322" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -22567,6 +23041,7 @@
         </is>
       </c>
       <c r="N323" t="inlineStr"/>
+      <c r="O323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -22635,6 +23110,7 @@
         </is>
       </c>
       <c r="N324" t="inlineStr"/>
+      <c r="O324" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -22703,6 +23179,7 @@
         </is>
       </c>
       <c r="N325" t="inlineStr"/>
+      <c r="O325" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -22771,6 +23248,7 @@
         </is>
       </c>
       <c r="N326" t="inlineStr"/>
+      <c r="O326" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -22839,6 +23317,7 @@
         </is>
       </c>
       <c r="N327" t="inlineStr"/>
+      <c r="O327" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -22907,6 +23386,7 @@
         </is>
       </c>
       <c r="N328" t="inlineStr"/>
+      <c r="O328" t="inlineStr"/>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -22975,6 +23455,7 @@
         </is>
       </c>
       <c r="N329" t="inlineStr"/>
+      <c r="O329" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -23043,6 +23524,7 @@
         </is>
       </c>
       <c r="N330" t="inlineStr"/>
+      <c r="O330" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -23111,6 +23593,7 @@
         </is>
       </c>
       <c r="N331" t="inlineStr"/>
+      <c r="O331" t="inlineStr"/>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -23179,6 +23662,7 @@
         </is>
       </c>
       <c r="N332" t="inlineStr"/>
+      <c r="O332" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -23247,6 +23731,7 @@
         </is>
       </c>
       <c r="N333" t="inlineStr"/>
+      <c r="O333" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -23315,6 +23800,7 @@
         </is>
       </c>
       <c r="N334" t="inlineStr"/>
+      <c r="O334" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -23383,6 +23869,7 @@
         </is>
       </c>
       <c r="N335" t="inlineStr"/>
+      <c r="O335" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -23451,6 +23938,7 @@
         </is>
       </c>
       <c r="N336" t="inlineStr"/>
+      <c r="O336" t="inlineStr"/>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -23523,6 +24011,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O337" t="inlineStr"/>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -23595,6 +24084,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O338" t="inlineStr"/>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -23667,6 +24157,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O339" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -23739,6 +24230,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O340" t="inlineStr"/>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -23811,6 +24303,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O341" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -23883,6 +24376,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O342" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -23955,6 +24449,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O343" t="inlineStr"/>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -24023,6 +24518,7 @@
         </is>
       </c>
       <c r="N344" t="inlineStr"/>
+      <c r="O344" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -24091,6 +24587,7 @@
         </is>
       </c>
       <c r="N345" t="inlineStr"/>
+      <c r="O345" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -24159,6 +24656,7 @@
         </is>
       </c>
       <c r="N346" t="inlineStr"/>
+      <c r="O346" t="inlineStr"/>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -24227,6 +24725,7 @@
         </is>
       </c>
       <c r="N347" t="inlineStr"/>
+      <c r="O347" t="inlineStr"/>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -24295,6 +24794,7 @@
         </is>
       </c>
       <c r="N348" t="inlineStr"/>
+      <c r="O348" t="inlineStr"/>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -24363,6 +24863,7 @@
         </is>
       </c>
       <c r="N349" t="inlineStr"/>
+      <c r="O349" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -24431,6 +24932,7 @@
         </is>
       </c>
       <c r="N350" t="inlineStr"/>
+      <c r="O350" t="inlineStr"/>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -24499,6 +25001,7 @@
         </is>
       </c>
       <c r="N351" t="inlineStr"/>
+      <c r="O351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -24567,6 +25070,7 @@
         </is>
       </c>
       <c r="N352" t="inlineStr"/>
+      <c r="O352" t="inlineStr"/>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -24635,6 +25139,7 @@
         </is>
       </c>
       <c r="N353" t="inlineStr"/>
+      <c r="O353" t="inlineStr"/>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -24703,6 +25208,7 @@
         </is>
       </c>
       <c r="N354" t="inlineStr"/>
+      <c r="O354" t="inlineStr"/>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -24771,6 +25277,7 @@
         </is>
       </c>
       <c r="N355" t="inlineStr"/>
+      <c r="O355" t="inlineStr"/>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -24839,6 +25346,7 @@
         </is>
       </c>
       <c r="N356" t="inlineStr"/>
+      <c r="O356" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -24907,6 +25415,7 @@
         </is>
       </c>
       <c r="N357" t="inlineStr"/>
+      <c r="O357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -24975,6 +25484,7 @@
         </is>
       </c>
       <c r="N358" t="inlineStr"/>
+      <c r="O358" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -25043,6 +25553,7 @@
         </is>
       </c>
       <c r="N359" t="inlineStr"/>
+      <c r="O359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -25111,6 +25622,7 @@
         </is>
       </c>
       <c r="N360" t="inlineStr"/>
+      <c r="O360" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -25179,6 +25691,7 @@
         </is>
       </c>
       <c r="N361" t="inlineStr"/>
+      <c r="O361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -25247,6 +25760,7 @@
         </is>
       </c>
       <c r="N362" t="inlineStr"/>
+      <c r="O362" t="inlineStr"/>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -25315,6 +25829,7 @@
         </is>
       </c>
       <c r="N363" t="inlineStr"/>
+      <c r="O363" t="inlineStr"/>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -25374,7 +25889,7 @@
       </c>
       <c r="L364" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M364" t="inlineStr">
@@ -25382,7 +25897,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N364" t="inlineStr"/>
+      <c r="N364" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O364" t="inlineStr"/>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -25442,7 +25962,7 @@
       </c>
       <c r="L365" t="inlineStr">
         <is>
-          <t>Not-Yet Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M365" t="inlineStr">
@@ -25450,7 +25970,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="N365" t="inlineStr"/>
+      <c r="N365" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="O365" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -25523,6 +26048,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O366" t="inlineStr"/>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -25595,6 +26121,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O367" t="inlineStr"/>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -25667,6 +26194,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O368" t="inlineStr"/>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -25739,6 +26267,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O369" t="inlineStr"/>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -25811,6 +26340,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O370" t="inlineStr"/>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -25883,6 +26413,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O371" t="inlineStr"/>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -25955,6 +26486,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O372" t="inlineStr"/>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
@@ -26027,6 +26559,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O373" t="inlineStr"/>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
@@ -26099,6 +26632,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O374" t="inlineStr"/>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
@@ -26171,6 +26705,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O375" t="inlineStr"/>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
@@ -26243,6 +26778,7 @@
           <t>done</t>
         </is>
       </c>
+      <c r="O376" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>